<commit_message>
feat: enhance country import with multilingual name support and add test files for validation
</commit_message>
<xml_diff>
--- a/test-excel-files/countries_test.xlsx
+++ b/test-excel-files/countries_test.xlsx
@@ -1,20 +1,20 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
-  </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties">
+  <Application>Microsoft Excel Compatible / Openpyxl 3.1.5</Application>
+  <AppVersion>3.1</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>openpyxl</dc:creator>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-28T00:49:15Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-28T00:49:15Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
   <fonts count="1">
@@ -124,7 +124,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -407,13 +407,28 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+  </sheets>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -427,6 +442,21 @@
           <t>name</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>nameEn</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>nameDe</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>nameFr</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -439,6 +469,21 @@
           <t>United States</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Vereinigte Staaten</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>États-Unis</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -451,6 +496,21 @@
           <t>Germany</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Allemagne</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -463,6 +523,21 @@
           <t>France</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Frankreich</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -475,6 +550,21 @@
           <t>Great Britain</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Great Britain</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Großbritannien</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Grande-Bretagne</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -487,6 +577,21 @@
           <t>Japan</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Japon</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -499,6 +604,21 @@
           <t>China</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Chine</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -511,6 +631,21 @@
           <t>Australia</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Australien</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Australie</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -523,6 +658,21 @@
           <t>Canada</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Kanada</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -535,6 +685,21 @@
           <t>Italy</t>
         </is>
       </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Italien</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Italie</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -545,6 +710,21 @@
       <c r="B11" t="inlineStr">
         <is>
           <t>Spain</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Spanien</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Espagne</t>
         </is>
       </c>
     </row>

</xml_diff>